<commit_message>
update excel and rule debt increase
</commit_message>
<xml_diff>
--- a/examples/excel/demo_scenarios.xlsx
+++ b/examples/excel/demo_scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cc1323\credit-assessment-system\examples\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548810F8-303B-4E9B-8AF1-8815CD168738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FBCA95-D1B0-4FAB-B16B-142B84B44F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="129">
   <si>
     <t>Credit Assessment System — Integrated Demo Scenario</t>
   </si>
@@ -415,6 +415,21 @@
   </si>
   <si>
     <t>production_value</t>
+  </si>
+  <si>
+    <t>bank_debt_current</t>
+  </si>
+  <si>
+    <t>bank_debt_1y_ago</t>
+  </si>
+  <si>
+    <t>bank_debt_2y_ago</t>
+  </si>
+  <si>
+    <t>bank_debt_3y_ago</t>
+  </si>
+  <si>
+    <t>bank_debt_4y_ago</t>
   </si>
 </sst>
 </file>
@@ -1307,7 +1322,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:AC2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1332,9 +1347,14 @@
     <col min="22" max="22" width="20" customWidth="1"/>
     <col min="23" max="23" width="18" customWidth="1"/>
     <col min="24" max="24" width="24" customWidth="1"/>
+    <col min="25" max="25" width="21.7109375" customWidth="1"/>
+    <col min="26" max="26" width="19.7109375" customWidth="1"/>
+    <col min="27" max="27" width="25.5703125" customWidth="1"/>
+    <col min="28" max="28" width="26" customWidth="1"/>
+    <col min="29" max="29" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1407,8 +1427,23 @@
       <c r="X1" s="3" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="2" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+      <c r="Y1" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -1478,6 +1513,21 @@
       </c>
       <c r="X2" s="6">
         <v>4800000</v>
+      </c>
+      <c r="Y2" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="Z2" s="5">
+        <v>800000</v>
+      </c>
+      <c r="AA2" s="5">
+        <v>800000</v>
+      </c>
+      <c r="AB2" s="5">
+        <v>800000</v>
+      </c>
+      <c r="AC2" s="5">
+        <v>800000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix tests excel and new rule
</commit_message>
<xml_diff>
--- a/examples/excel/demo_scenarios.xlsx
+++ b/examples/excel/demo_scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cc1323\credit-assessment-system\examples\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FBCA95-D1B0-4FAB-B16B-142B84B44F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546646C9-65F5-482B-92E7-FA047E7B05DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="134">
   <si>
     <t>Credit Assessment System — Integrated Demo Scenario</t>
   </si>
@@ -430,6 +430,21 @@
   </si>
   <si>
     <t>bank_debt_4y_ago</t>
+  </si>
+  <si>
+    <t>trade_payables_current</t>
+  </si>
+  <si>
+    <t>trade_payables_1y_ago</t>
+  </si>
+  <si>
+    <t>trade_payables_2y_ago</t>
+  </si>
+  <si>
+    <t>trade_payables_3y_ago</t>
+  </si>
+  <si>
+    <t>trade_payables_4y_ago</t>
   </si>
 </sst>
 </file>
@@ -1322,7 +1337,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1352,9 +1367,10 @@
     <col min="27" max="27" width="25.5703125" customWidth="1"/>
     <col min="28" max="28" width="26" customWidth="1"/>
     <col min="29" max="29" width="24" customWidth="1"/>
+    <col min="30" max="34" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1442,8 +1458,23 @@
       <c r="AC1" s="3" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="2" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+      <c r="AD1" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="AG1" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="AH1" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:34" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -1527,6 +1558,21 @@
         <v>800000</v>
       </c>
       <c r="AC2" s="5">
+        <v>800000</v>
+      </c>
+      <c r="AD2" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="AE2" s="5">
+        <v>800000</v>
+      </c>
+      <c r="AF2" s="5">
+        <v>800000</v>
+      </c>
+      <c r="AG2" s="5">
+        <v>800000</v>
+      </c>
+      <c r="AH2" s="5">
         <v>800000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix excel and new rule tax
</commit_message>
<xml_diff>
--- a/examples/excel/demo_scenarios.xlsx
+++ b/examples/excel/demo_scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cc1323\credit-assessment-system\examples\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE56F73-8D2A-4A33-A8DF-C73F8296D09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D332B0A-ED21-4524-BBB1-64F8BE6720A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="141">
   <si>
     <t>Credit Assessment System — Integrated Demo Scenario</t>
   </si>
@@ -460,6 +460,12 @@
   </si>
   <si>
     <t>avg_payment_days_4y_ago</t>
+  </si>
+  <si>
+    <t>tax_debt</t>
+  </si>
+  <si>
+    <t>total_liabilities</t>
   </si>
 </sst>
 </file>
@@ -1352,7 +1358,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AM2"/>
+  <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1384,9 +1390,10 @@
     <col min="29" max="29" width="24" customWidth="1"/>
     <col min="30" max="34" width="23" customWidth="1"/>
     <col min="35" max="39" width="28.28515625" customWidth="1"/>
+    <col min="40" max="41" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:41" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1504,8 +1511,14 @@
       <c r="AM1" s="3" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="2" spans="1:39" ht="45" x14ac:dyDescent="0.25">
+      <c r="AN1" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AO1" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:41" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -1620,6 +1633,12 @@
       </c>
       <c r="AM2" s="5">
         <v>70</v>
+      </c>
+      <c r="AN2" s="5">
+        <v>20000</v>
+      </c>
+      <c r="AO2" s="5">
+        <v>100000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update rule avg collection
</commit_message>
<xml_diff>
--- a/examples/excel/demo_scenarios.xlsx
+++ b/examples/excel/demo_scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cc1323\credit-assessment-system\examples\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D332B0A-ED21-4524-BBB1-64F8BE6720A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7609DB-539C-4917-AB20-9222E62ABB15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="146">
   <si>
     <t>Credit Assessment System — Integrated Demo Scenario</t>
   </si>
@@ -466,6 +466,21 @@
   </si>
   <si>
     <t>total_liabilities</t>
+  </si>
+  <si>
+    <t>avg_collection_days_current</t>
+  </si>
+  <si>
+    <t>avg_collection_days_1y_ago</t>
+  </si>
+  <si>
+    <t>avg_collection_days_2y_ago</t>
+  </si>
+  <si>
+    <t>avg_collection_days_3y_ago</t>
+  </si>
+  <si>
+    <t>avg_collection_days_4y_ago</t>
   </si>
 </sst>
 </file>
@@ -1358,7 +1373,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AO2"/>
+  <dimension ref="A1:AT2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1391,9 +1406,12 @@
     <col min="30" max="34" width="23" customWidth="1"/>
     <col min="35" max="39" width="28.28515625" customWidth="1"/>
     <col min="40" max="41" width="20.28515625" customWidth="1"/>
+    <col min="42" max="42" width="27.5703125" customWidth="1"/>
+    <col min="43" max="43" width="24.7109375" customWidth="1"/>
+    <col min="44" max="46" width="19.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:46" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1517,8 +1535,23 @@
       <c r="AO1" s="3" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="2" spans="1:41" ht="45" x14ac:dyDescent="0.25">
+      <c r="AP1" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AQ1" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AR1" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="AS1" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="AT1" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:46" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -1639,6 +1672,21 @@
       </c>
       <c r="AO2" s="5">
         <v>100000</v>
+      </c>
+      <c r="AP2" s="5">
+        <v>120</v>
+      </c>
+      <c r="AQ2" s="5">
+        <v>110</v>
+      </c>
+      <c r="AR2" s="5">
+        <v>90</v>
+      </c>
+      <c r="AS2" s="5">
+        <v>80</v>
+      </c>
+      <c r="AT2" s="5">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>